<commit_message>
Regenerate analysis outputs in data/
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/guests_junk.xlsx
+++ b/data/guests_junk.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,56 +413,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>party</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>uid</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Talkshow</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>validation_status</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>validation_reason</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>name_clean</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>reject_reason</t>
         </is>
@@ -483,7 +471,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Vizepräsidentin des Deutschen Bundestages</t>
+          <t>im Bundestag</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -491,31 +479,31 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>db_SJGJJ</t>
+          <t>xYzH9-qg</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Anne Will - 11.01.2009</t>
+          <t>Anne Will - 02.02.2020</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Vizepräsidentin des Deutschen Bundestages</t>
+          <t>im Bundestag</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>contains_junk_phrase_words</t>
+          <t>contains_role_word</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>im Bundestag</t>
+          <t>Mitglied des Bundestages</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -523,19 +511,19 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>xYzH9-qg</t>
+          <t>AvH4dHBQ</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Anne Will - 02.02.2020</t>
+          <t>Anne Will - 17.09.2023</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>im Bundestag</t>
+          <t>Mitglied des Bundestages</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -547,99 +535,107 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mitglied des Bundestages</t>
+          <t>Gäste</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Innenminister Nordrhein-Westfalen</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Hinweis zum DatenschutzMit Klick auf "Einverstanden" können Sie diese Seite in sozialen Netzwerken weiterempfehlen. Dabei besteht die Möglichkeit, dass Daten von Ihrem Computer zum jeweiligen Anbieter sowie Daten des Anbieters auf Ihren Computer übertragen werden. Diese Zustimmung wird von Ihnen für 24 Stunden erteilt.</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AvH4dHBQ</t>
+          <t>qvqZ1pfC</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Anne Will - 17.09.2023</t>
+          <t>Caren Miosga - 25.08.2024</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Mitglied des Bundestages</t>
+          <t>Gäste</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>contains_role_word</t>
+          <t>contains_junk_phrase_words</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Journalist</t>
+          <t>FDP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Autor des Buches „Der Baader-Meinhof-Komplex“</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Autor des Buches „Der Baader-Meinhof-Komplex“</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7anKhM02</t>
+          <t>jqfhqThD</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Anne Will - 21.09.2008</t>
+          <t>hart aber fair - 22.08.2022</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Journalist</t>
+          <t>FDP</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>contains_role_word</t>
+          <t>party_or_org_token</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>„dbb beamtenbund</t>
+          <t>Fraktionsvorsitzender; Mitglied des Präsidiums</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Christian Dürr</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Christian Dürr</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>LdAZfFoi</t>
+          <t>jqfhqThD</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Anne Will - 31.01.2010</t>
+          <t>hart aber fair - 22.08.2022</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>„dbb beamtenbund</t>
+          <t>Fraktionsvorsitzender; Mitglied des Präsidiums</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -651,7 +647,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fachbereich Gesundheit</t>
+          <t>Die Linke</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -659,59 +655,59 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>I5TF5_eB</t>
+          <t>jqfhqThD</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Anne Will - 08.03.2009</t>
+          <t>hart aber fair - 22.08.2022</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Fachbereich Gesundheit</t>
+          <t>Die Linke</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>contains_junk_phrase_words</t>
+          <t>party_or_org_token</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gäste</t>
+          <t>Direktor des Instituts der deutschen Wirtschaft Köln</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Innenminister Nordrhein-Westfalen</t>
+          <t>Michael Hüther</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hinweis zum DatenschutzMit Klick auf "Einverstanden" können Sie diese Seite in sozialen Netzwerken weiterempfehlen. Dabei besteht die Möglichkeit, dass Daten von Ihrem Computer zum jeweiligen Anbieter sowie Daten des Anbieters auf Ihren Computer übertragen werden. Diese Zustimmung wird von Ihnen für 24 Stunden erteilt.</t>
+          <t>Michael Hüther</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>qvqZ1pfC</t>
+          <t>jqfhqThD</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Caren Miosga - 25.08.24</t>
+          <t>hart aber fair - 22.08.2022</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Gäste</t>
+          <t>Direktor des Instituts der deutschen Wirtschaft Köln</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -723,7 +719,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Familie Frauen</t>
+          <t>B’90</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -731,31 +727,31 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>DAQqc733</t>
+          <t>ox2YsqDq</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>hart aber fair - 13.09.2006</t>
+          <t>maischberger - 19.03.2024</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Familie Frauen</t>
+          <t>B'90</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>contains_junk_phrase_words</t>
+          <t>too_short_token</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Expertin für Islam</t>
+          <t>Grüne</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -763,31 +759,31 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>aU_2KMoS</t>
+          <t>ox2YsqDq</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>hart aber fair - 07.10.2009</t>
+          <t>maischberger - 19.03.2024</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Expertin für Islam</t>
+          <t>Grüne</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>contains_role_word</t>
+          <t>party_or_org_token</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FDP</t>
+          <t>CSU</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -795,19 +791,19 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>jqfhqThD</t>
+          <t>ox2YsqDq</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>hart aber fair - 22.08.2022</t>
+          <t>maischberger - 19.03.2024</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>FDP</t>
+          <t>CSU</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -819,67 +815,67 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fraktionsvorsitzender; Mitglied des Präsidiums</t>
+          <t>Vincent productions GmbH.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Christian Dürr</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Christian Dürr</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>jqfhqThD</t>
+          <t>ox2YsqDq</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>hart aber fair - 22.08.2022</t>
+          <t>maischberger - 19.03.2024</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Fraktionsvorsitzender; Mitglied des Präsidiums</t>
+          <t>Vincent productions GmbH.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>contains_role_word</t>
+          <t>org_pattern_found</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Die Linke</t>
+          <t>FDP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Bundestagsvizepräsident</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Bundestagsvizepräsident</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>jqfhqThD</t>
+          <t>pMlMm9w9</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>hart aber fair - 22.08.2022</t>
+          <t>maischberger - 12.10.2022</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Die Linke</t>
+          <t>FDP</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -891,111 +887,119 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Direktor des Instituts der deutschen Wirtschaft Köln</t>
+          <t>Bundesfinanzminister</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Michael Hüther</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Michael Hüther</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>jqfhqThD</t>
+          <t>cmojDYvR</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>hart aber fair - 22.08.2022</t>
+          <t>maischberger - 12.08.2020</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Direktor des Instituts der deutschen Wirtschaft Köln</t>
+          <t>Bundesfinanzminister</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>contains_junk_phrase_words</t>
+          <t>contains_role_word</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>B’90</t>
+          <t>ehemaliger Bundesinnenminister</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Hazar Abaza</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Hazar Abaza</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ox2YsqDq</t>
+          <t>cmojDYvR</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>maischberger - 19.03.2024</t>
+          <t>maischberger - 12.08.2020</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>B'90</t>
+          <t>ehemaliger Bundesinnenminister</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>too_short_token</t>
+          <t>contains_junk_phrase_words</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Grüne</t>
+          <t>Abiturientin; floh 2015 aus Syrien</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Hans Rudolf Wöhrl</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Hans Rudolf Wöhrl</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ox2YsqDq</t>
+          <t>cmojDYvR</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>maischberger - 19.03.2024</t>
+          <t>maischberger - 12.08.2020</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Grüne</t>
+          <t>Abiturientin; floh 2015 aus Syrien</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>party_or_org_token</t>
+          <t>contains_junk_phrase_words</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CSU</t>
+          <t>Moderatorin ARD-„Morgenmagazin“</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -1003,31 +1007,31 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ox2YsqDq</t>
+          <t>cmojDYvR</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>maischberger - 19.03.2024</t>
+          <t>maischberger - 12.08.2020</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>CSU</t>
+          <t>Moderatorin ARD-„Morgenmagazin"</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>party_or_org_token</t>
+          <t>contains_role_word</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Vincent productions GmbH.</t>
+          <t>Unternehmer</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -1035,31 +1039,31 @@
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ox2YsqDq</t>
+          <t>cmojDYvR</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>maischberger - 19.03.2024</t>
+          <t>maischberger - 12.08.2020</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Vincent productions GmbH.</t>
+          <t>Unternehmer</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>org_pattern_found</t>
+          <t>contains_role_word</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>seine Frau Liselotte</t>
+          <t>CSU</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -1067,59 +1071,51 @@
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>NFK4zZ1X</t>
+          <t>FPI41BOT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>maischberger - 22.04.2008</t>
+          <t>maischberger - 28.03.2023</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>seine Frau Liselotte</t>
+          <t>CSU</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>contains_junk_phrase_words</t>
+          <t>party_or_org_token</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FDP</t>
+          <t>Die Linke</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Bundestagsvizepräsident</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Bundestagsvizepräsident</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>pMlMm9w9</t>
+          <t>FPI41BOT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>maischberger - 12.10.2022</t>
+          <t>maischberger - 28.03.2023</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>FDP</t>
+          <t>Die Linke</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1131,7 +1127,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bundesfinanzminister</t>
+          <t>Vincent productions GmbH.</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1139,99 +1135,99 @@
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>cmojDYvR</t>
+          <t>FPI41BOT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>maischberger - 12.08.2020</t>
+          <t>maischberger - 28.03.2023</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Bundesfinanzminister</t>
+          <t>Vincent productions GmbH.</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>contains_role_word</t>
+          <t>org_pattern_found</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ehemaliger Bundesinnenminister</t>
+          <t>Bundesvorsitzender der Jungen Union</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Hazar Abaza</t>
+          <t>JU)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Hazar Abaza</t>
+          <t>JU)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>cmojDYvR</t>
+          <t>y_UtLThE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>maischberger - 12.08.2020</t>
+          <t>Maybrit Illner - 19.05.2016</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>ehemaliger Bundesinnenminister</t>
+          <t>Bundesvorsitzender der Jungen Union</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>contains_junk_phrase_words</t>
+          <t>contains_role_word</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Abiturientin; floh 2015 aus Syrien</t>
+          <t>Familie Pinzler</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hans Rudolf Wöhrl</t>
+          <t>hat versucht ein Jahr konsequent CO2 zu vermeiden</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Hans Rudolf Wöhrl</t>
+          <t>hat versucht ein Jahr konsequent CO2 zu vermeiden</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>cmojDYvR</t>
+          <t>L6ft1_3u</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>maischberger - 12.08.2020</t>
+          <t>Maybrit Illner - 23.08.2018</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Abiturientin; floh 2015 aus Syrien</t>
+          <t>Familie Pinzler</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1243,7 +1239,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Moderatorin ARD-„Morgenmagazin“</t>
+          <t>Autor u. a. „Al-Qaidas deutsche Kämpfer</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -1251,294 +1247,22 @@
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>cmojDYvR</t>
+          <t>lGWMBDxs</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>maischberger - 12.08.2020</t>
+          <t>Maybrit Illner - 22.01.2015</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Moderatorin ARD-„Morgenmagazin"</t>
+          <t>Autor u. a. „Al-Qaidas deutsche Kämpfer</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
-        <is>
-          <t>contains_role_word</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Unternehmer</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>cmojDYvR</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>maischberger - 12.08.2020</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Unternehmer</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>contains_role_word</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Altersforscher</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>KKP4lr0S</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>maischberger - 02.02.2010</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Altersforscher</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>contains_role_word</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>CSU</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>FPI41BOT</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>maischberger - 28.03.2023</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>CSU</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>party_or_org_token</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Die Linke</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>FPI41BOT</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>maischberger - 28.03.2023</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Die Linke</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>party_or_org_token</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Vincent productions GmbH.</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>FPI41BOT</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>maischberger - 28.03.2023</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Vincent productions GmbH.</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>org_pattern_found</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Bundesvorsitzender der Jungen Union</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>JU)</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>JU)</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>y_UtLThE</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Maybrit Illner - 19.05.2016</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Bundesvorsitzender der Jungen Union</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>contains_role_word</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Familie Pinzler</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>hat versucht ein Jahr konsequent CO2 zu vermeiden</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>hat versucht ein Jahr konsequent CO2 zu vermeiden</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>L6ft1_3u</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Maybrit Illner - 23.08.2018</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Familie Pinzler</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>contains_junk_phrase_words</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Autor u. a. „Al-Qaidas deutsche Kämpfer</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>lGWMBDxs</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Maybrit Illner - 22.01.2015</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Autor u. a. „Al-Qaidas deutsche Kämpfer</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
         <is>
           <t>contains_role_word</t>
         </is>

</xml_diff>